<commit_message>
fixes read me and metadata
</commit_message>
<xml_diff>
--- a/templates/metadata_turbo_id.xlsx
+++ b/templates/metadata_turbo_id.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nropek/Dropbox (Dropbox @RU)/TurboID manuscript/Mass-spectrometry datasets/02_metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6FC405C-A4E7-CC4A-880F-53AC0A9D6B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86BE6DBC-A004-4C4E-A5F4-9FD4BAA962F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="44160" windowHeight="20760" activeTab="3" xr2:uid="{FE8B76B0-690F-4941-9173-C8E6A2A99654}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="27120" windowHeight="16520" activeTab="3" xr2:uid="{FE8B76B0-690F-4941-9173-C8E6A2A99654}"/>
   </bookViews>
   <sheets>
     <sheet name="Files" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="887" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="267">
   <si>
     <t>Abbreviation</t>
   </si>
@@ -753,9 +753,6 @@
     <t>5) cd \Users\Public</t>
   </si>
   <si>
-    <t xml:space="preserve">6) .\start_pipeline.ps1 process file folder </t>
-  </si>
-  <si>
     <t xml:space="preserve">8) Copy, paste conditions_metadata.csv and metadata_col.csv into the folder you just created/01_processed_files (you can compy them from gitlab/turboid/templates, or from old processing folders) </t>
   </si>
   <si>
@@ -783,12 +780,6 @@
     <t xml:space="preserve">17) wait until you see goodbye message </t>
   </si>
   <si>
-    <t>1*</t>
-  </si>
-  <si>
-    <t>note: if you are requested to run 2 pep per protein, repeat the census out processing and enter 2 in this field, make sure to label the results folder correctly when the program asks you</t>
-  </si>
-  <si>
     <t xml:space="preserve">STEP 1: Census-out processing </t>
   </si>
   <si>
@@ -820,6 +811,33 @@
   </si>
   <si>
     <t xml:space="preserve">14) wait until you see the goodbye message </t>
+  </si>
+  <si>
+    <t>fast_turbo(+)_4</t>
+  </si>
+  <si>
+    <t>census-out_EV2-45_BasalvsFastingvsLPS_CD19_F_Plasma_16plex</t>
+  </si>
+  <si>
+    <t>EV2-45</t>
+  </si>
+  <si>
+    <t>CD19 (females)</t>
+  </si>
+  <si>
+    <t>EV2-47</t>
+  </si>
+  <si>
+    <t>CD19 (males)</t>
+  </si>
+  <si>
+    <t>???</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6) .\start_pipeline.ps1 process_file_folder </t>
+  </si>
+  <si>
+    <t>*note: if you are requested to run 2 pep per protein, repeat the census out processing and enter 2 in this field, make sure to label the results folder correctly when the program asks you</t>
   </si>
 </sst>
 </file>
@@ -915,6 +933,7 @@
     </font>
     <font>
       <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1023,7 +1042,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1096,23 +1115,30 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1125,10 +1151,22 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1137,27 +1175,12 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1169,18 +1192,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1355,15 +1366,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>411630</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>1</xdr:row>
-          <xdr:rowOff>222624</xdr:rowOff>
+          <xdr:rowOff>228600</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>95624</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>3</xdr:row>
-          <xdr:rowOff>92636</xdr:rowOff>
+          <xdr:rowOff>88900</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1373,7 +1384,7 @@
                   <a14:compatExt spid="_x0000_s4099"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CA9EE10D-E6D5-794C-9F32-18C406C1EAF4}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000003100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1422,15 +1433,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>401918</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>2</xdr:row>
-          <xdr:rowOff>135964</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>97118</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>97864</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1440,7 +1451,7 @@
                   <a14:compatExt spid="_x0000_s4100"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{15789946-9C82-A645-9068-7C07476C2DE5}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000004100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1489,15 +1500,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>394447</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>3</xdr:row>
-          <xdr:rowOff>133724</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>89647</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>5</xdr:row>
-          <xdr:rowOff>95624</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1507,7 +1518,7 @@
                   <a14:compatExt spid="_x0000_s4101"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{022E9AD9-C9DC-474A-A0A4-23E64143A4FD}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000005100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1556,15 +1567,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396689</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>141194</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91889</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>6</xdr:row>
-          <xdr:rowOff>103094</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1574,7 +1585,7 @@
                   <a14:compatExt spid="_x0000_s4102"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A4CA8351-DEFF-6446-970F-2EF7271741D8}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000006100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1623,15 +1634,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396689</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>5</xdr:row>
-          <xdr:rowOff>141194</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91889</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>7</xdr:row>
-          <xdr:rowOff>103094</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1641,7 +1652,7 @@
                   <a14:compatExt spid="_x0000_s4103"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F59BF483-63F4-7743-8C5E-967485791537}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000007100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1690,15 +1701,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396689</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>6</xdr:row>
-          <xdr:rowOff>133724</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91889</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>8</xdr:row>
-          <xdr:rowOff>95624</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1708,7 +1719,7 @@
                   <a14:compatExt spid="_x0000_s4104"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0A373BA-5DFE-2D4B-9E95-EC845160B86F}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000008100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1757,15 +1768,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396688</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>7</xdr:row>
-          <xdr:rowOff>133724</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91888</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>9</xdr:row>
-          <xdr:rowOff>95624</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1775,7 +1786,7 @@
                   <a14:compatExt spid="_x0000_s4105"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{324E7085-B268-504F-8D55-3346EAAF00EE}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000009100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1826,13 +1837,13 @@
           <xdr:col>0</xdr:col>
           <xdr:colOff>393700</xdr:colOff>
           <xdr:row>9</xdr:row>
-          <xdr:rowOff>117289</xdr:rowOff>
+          <xdr:rowOff>114300</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
           <xdr:colOff>88900</xdr:colOff>
           <xdr:row>11</xdr:row>
-          <xdr:rowOff>79189</xdr:rowOff>
+          <xdr:rowOff>76200</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1842,7 +1853,7 @@
                   <a14:compatExt spid="_x0000_s4106"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{88D30BE6-4067-B148-BC33-8914C49CB8BB}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000A100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1891,15 +1902,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>404159</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>10</xdr:row>
-          <xdr:rowOff>130736</xdr:rowOff>
+          <xdr:rowOff>127000</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>99359</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>12</xdr:row>
-          <xdr:rowOff>92636</xdr:rowOff>
+          <xdr:rowOff>88900</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1909,7 +1920,7 @@
                   <a14:compatExt spid="_x0000_s4107"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF01BB4B-AFB7-0446-9DC8-9DE71EC626AB}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000B100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1958,15 +1969,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>401918</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>11</xdr:row>
-          <xdr:rowOff>128494</xdr:rowOff>
+          <xdr:rowOff>127000</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>97118</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>13</xdr:row>
-          <xdr:rowOff>90394</xdr:rowOff>
+          <xdr:rowOff>88900</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1976,7 +1987,7 @@
                   <a14:compatExt spid="_x0000_s4108"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{159E8957-9CD7-8143-B1A7-707866496962}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000C100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2025,15 +2036,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>401918</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>12</xdr:row>
-          <xdr:rowOff>143436</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>97118</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>14</xdr:row>
-          <xdr:rowOff>105336</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2043,7 +2054,7 @@
                   <a14:compatExt spid="_x0000_s4109"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF2CD9BA-6CD0-2E45-8531-B7480FCDB085}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000D100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2092,15 +2103,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>394448</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>13</xdr:row>
-          <xdr:rowOff>133724</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>89648</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>15</xdr:row>
-          <xdr:rowOff>95624</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2110,7 +2121,7 @@
                   <a14:compatExt spid="_x0000_s4110"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6F8B439F-09F3-894F-93C3-1B61D9F374B2}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000E100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2159,15 +2170,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>404158</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>14</xdr:row>
-          <xdr:rowOff>141194</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>99358</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>16</xdr:row>
-          <xdr:rowOff>103094</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2177,7 +2188,7 @@
                   <a14:compatExt spid="_x0000_s4111"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AC7C0281-A330-9E4F-9A23-AE5FA38DDCB4}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000F100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2226,15 +2237,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>401918</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>15</xdr:row>
-          <xdr:rowOff>141194</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>97118</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>17</xdr:row>
-          <xdr:rowOff>103094</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2244,7 +2255,7 @@
                   <a14:compatExt spid="_x0000_s4112"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9ED98A50-22EB-144F-BEA7-ECFCD7419907}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000010100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2293,15 +2304,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>394447</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>16</xdr:row>
-          <xdr:rowOff>133723</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>89647</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>18</xdr:row>
-          <xdr:rowOff>95623</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2311,7 +2322,7 @@
                   <a14:compatExt spid="_x0000_s4113"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{32B1E6D8-7579-1646-BDA7-C6EA8FC680DF}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000011100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2360,15 +2371,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396688</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>17</xdr:row>
-          <xdr:rowOff>133724</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91888</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>19</xdr:row>
-          <xdr:rowOff>95624</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2378,7 +2389,7 @@
                   <a14:compatExt spid="_x0000_s4114"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0C9D2DE0-B4FA-784E-AB41-A37B756876F7}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000012100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2427,15 +2438,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396688</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>18</xdr:row>
-          <xdr:rowOff>141194</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91888</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>20</xdr:row>
-          <xdr:rowOff>103094</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2445,7 +2456,7 @@
                   <a14:compatExt spid="_x0000_s4115"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AAF614D2-CD5E-2343-A2E5-EE8433E4FC2D}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000013100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2494,15 +2505,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396689</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>19</xdr:row>
-          <xdr:rowOff>133724</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91889</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>21</xdr:row>
-          <xdr:rowOff>95624</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2512,7 +2523,7 @@
                   <a14:compatExt spid="_x0000_s4116"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B6C977B-67E5-A34A-9DB9-8D2DB6ED7A65}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000014100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2561,15 +2572,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>404159</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>20</xdr:row>
-          <xdr:rowOff>141194</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>99359</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>22</xdr:row>
-          <xdr:rowOff>103094</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2579,7 +2590,7 @@
                   <a14:compatExt spid="_x0000_s4117"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FBD646E9-2F73-0B4B-B864-C18E21FC0460}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000015100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2628,15 +2639,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>401917</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>23</xdr:row>
-          <xdr:rowOff>118782</xdr:rowOff>
+          <xdr:rowOff>114300</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>97117</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>25</xdr:row>
-          <xdr:rowOff>80682</xdr:rowOff>
+          <xdr:rowOff>76200</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2646,7 +2657,7 @@
                   <a14:compatExt spid="_x0000_s4118"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEF701B3-B441-534D-9705-9EC8A4E6E71E}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000016100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2695,15 +2706,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>416859</xdr:colOff>
+          <xdr:colOff>419100</xdr:colOff>
           <xdr:row>26</xdr:row>
-          <xdr:rowOff>227853</xdr:rowOff>
+          <xdr:rowOff>228600</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>112059</xdr:colOff>
+          <xdr:colOff>114300</xdr:colOff>
           <xdr:row>28</xdr:row>
-          <xdr:rowOff>85164</xdr:rowOff>
+          <xdr:rowOff>88900</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2713,7 +2724,7 @@
                   <a14:compatExt spid="_x0000_s4119"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{10755970-3D92-D749-A910-4A7A31E075B6}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000017100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2762,15 +2773,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>407148</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>27</xdr:row>
-          <xdr:rowOff>135964</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>102348</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>29</xdr:row>
-          <xdr:rowOff>97864</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2780,7 +2791,7 @@
                   <a14:compatExt spid="_x0000_s4120"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B21057FC-F46B-F743-9C35-F3D7A22A7AA3}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000018100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2829,15 +2840,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>401917</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>28</xdr:row>
-          <xdr:rowOff>126253</xdr:rowOff>
+          <xdr:rowOff>127000</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>97117</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>30</xdr:row>
-          <xdr:rowOff>88153</xdr:rowOff>
+          <xdr:rowOff>88900</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2847,7 +2858,7 @@
                   <a14:compatExt spid="_x0000_s4121"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E1ECF64-6916-F04A-901E-4058222C8634}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000019100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2896,15 +2907,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>394447</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>29</xdr:row>
-          <xdr:rowOff>135965</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>89647</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>31</xdr:row>
-          <xdr:rowOff>97865</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2914,7 +2925,7 @@
                   <a14:compatExt spid="_x0000_s4122"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6FC9643D-D01A-4641-B4D1-313FF1E2348B}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00001A100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2963,15 +2974,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396688</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>30</xdr:row>
-          <xdr:rowOff>133723</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91888</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>32</xdr:row>
-          <xdr:rowOff>95623</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2981,7 +2992,7 @@
                   <a14:compatExt spid="_x0000_s4123"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42CDCC78-8C97-6246-8008-1F887CE00BF9}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00001B100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3030,15 +3041,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396688</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>31</xdr:row>
-          <xdr:rowOff>126253</xdr:rowOff>
+          <xdr:rowOff>127000</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91888</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>33</xdr:row>
-          <xdr:rowOff>119529</xdr:rowOff>
+          <xdr:rowOff>114300</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3048,7 +3059,7 @@
                   <a14:compatExt spid="_x0000_s4124"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBD652D4-4A2F-0A40-BC69-D9438FED02AD}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00001C100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3097,15 +3108,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396689</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>32</xdr:row>
-          <xdr:rowOff>135964</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91889</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>34</xdr:row>
-          <xdr:rowOff>123264</xdr:rowOff>
+          <xdr:rowOff>127000</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3115,7 +3126,7 @@
                   <a14:compatExt spid="_x0000_s4125"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F49A1BB1-D902-5D40-B33D-2FA43EAAC685}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00001D100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3164,15 +3175,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396688</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>33</xdr:row>
-          <xdr:rowOff>133724</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91888</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>35</xdr:row>
-          <xdr:rowOff>121024</xdr:rowOff>
+          <xdr:rowOff>127000</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3182,7 +3193,7 @@
                   <a14:compatExt spid="_x0000_s4126"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3193B2B5-D39A-F34D-80D2-81627E674C10}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00001E100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3231,15 +3242,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396688</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>34</xdr:row>
-          <xdr:rowOff>133724</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>91888</xdr:colOff>
+          <xdr:colOff>88900</xdr:colOff>
           <xdr:row>36</xdr:row>
-          <xdr:rowOff>121024</xdr:rowOff>
+          <xdr:rowOff>127000</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3249,7 +3260,7 @@
                   <a14:compatExt spid="_x0000_s4127"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3BC4000F-0F07-D74F-BDDC-C4CCC0499AEC}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00001F100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3298,15 +3309,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>404159</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>35</xdr:row>
-          <xdr:rowOff>126253</xdr:rowOff>
+          <xdr:rowOff>127000</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>99359</xdr:colOff>
+          <xdr:colOff>101600</xdr:colOff>
           <xdr:row>37</xdr:row>
-          <xdr:rowOff>113553</xdr:rowOff>
+          <xdr:rowOff>114300</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3316,7 +3327,7 @@
                   <a14:compatExt spid="_x0000_s4128"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8BC21280-30F1-144F-BC31-3C5D003D7CD1}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000020100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3362,14 +3373,19 @@
   </mc:AlternateContent>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
+      <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>401917</xdr:colOff>
+          <xdr:colOff>406400</xdr:colOff>
           <xdr:row>38</xdr:row>
-          <xdr:rowOff>126253</xdr:rowOff>
+          <xdr:rowOff>127000</xdr:rowOff>
         </xdr:from>
-        <xdr:ext cx="382494" cy="365312"/>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>101600</xdr:colOff>
+          <xdr:row>40</xdr:row>
+          <xdr:rowOff>88900</xdr:rowOff>
+        </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4129" name="Check Box 33" hidden="1">
@@ -3378,7 +3394,7 @@
                   <a14:compatExt spid="_x0000_s4129"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69CAEAE7-BC9A-474E-82EA-708131EF651A}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000021100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3418,20 +3434,25 @@
           </xdr:spPr>
         </xdr:sp>
         <xdr:clientData/>
-      </xdr:oneCellAnchor>
+      </xdr:twoCellAnchor>
     </mc:Choice>
     <mc:Fallback/>
   </mc:AlternateContent>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
+      <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396688</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>39</xdr:row>
-          <xdr:rowOff>133723</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
-        <xdr:ext cx="382494" cy="365312"/>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>88900</xdr:colOff>
+          <xdr:row>41</xdr:row>
+          <xdr:rowOff>101600</xdr:rowOff>
+        </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4130" name="Check Box 34" hidden="1">
@@ -3440,7 +3461,7 @@
                   <a14:compatExt spid="_x0000_s4130"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D0C6304-F84B-F64D-BEDB-41720F1C96D1}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000022100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3480,7 +3501,7 @@
           </xdr:spPr>
         </xdr:sp>
         <xdr:clientData/>
-      </xdr:oneCellAnchor>
+      </xdr:twoCellAnchor>
     </mc:Choice>
     <mc:Fallback/>
   </mc:AlternateContent>
@@ -3489,15 +3510,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>398930</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>37</xdr:row>
           <xdr:rowOff>215900</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>14942</xdr:colOff>
+          <xdr:colOff>12700</xdr:colOff>
           <xdr:row>39</xdr:row>
-          <xdr:rowOff>85912</xdr:rowOff>
+          <xdr:rowOff>88900</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3507,7 +3528,7 @@
                   <a14:compatExt spid="_x0000_s4133"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E0D5A344-8A05-314B-AE5C-F5B5D4621454}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000025100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3546,7 +3567,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="32004" rIns="0" bIns="32004" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -3581,14 +3602,19 @@
   </mc:AlternateContent>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
+      <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>396688</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>40</xdr:row>
-          <xdr:rowOff>126253</xdr:rowOff>
+          <xdr:rowOff>127000</xdr:rowOff>
         </xdr:from>
-        <xdr:ext cx="382494" cy="396688"/>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>88900</xdr:colOff>
+          <xdr:row>42</xdr:row>
+          <xdr:rowOff>114300</xdr:rowOff>
+        </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4134" name="Check Box 38" hidden="1">
@@ -3597,7 +3623,7 @@
                   <a14:compatExt spid="_x0000_s4134"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA4127C0-CD7D-1B4C-B790-B0A987E461F4}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000026100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3637,7 +3663,7 @@
           </xdr:spPr>
         </xdr:sp>
         <xdr:clientData/>
-      </xdr:oneCellAnchor>
+      </xdr:twoCellAnchor>
     </mc:Choice>
     <mc:Fallback/>
   </mc:AlternateContent>
@@ -3646,15 +3672,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>395941</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>41</xdr:row>
-          <xdr:rowOff>141941</xdr:rowOff>
+          <xdr:rowOff>139700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>7471</xdr:colOff>
+          <xdr:colOff>12700</xdr:colOff>
           <xdr:row>43</xdr:row>
-          <xdr:rowOff>116541</xdr:rowOff>
+          <xdr:rowOff>114300</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3664,7 +3690,7 @@
                   <a14:compatExt spid="_x0000_s4135"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{86293271-2714-5C41-BAEF-99879C927127}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000027100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -4285,31 +4311,30 @@
       <c r="G12" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="H12" s="40" t="s">
+      <c r="H12" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="42" t="s">
+      <c r="A13" t="s">
         <v>166</v>
       </c>
-      <c r="B13" s="42" t="s">
+      <c r="B13" t="s">
         <v>165</v>
       </c>
-      <c r="C13" s="41" t="s">
+      <c r="C13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="42">
+      <c r="D13">
         <v>16</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="41" t="s">
+      <c r="F13" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="G13" s="41" t="s">
+      <c r="G13" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="H13" s="41" t="s">
+      <c r="H13" s="2" t="s">
         <v>231</v>
       </c>
     </row>
@@ -4329,7 +4354,7 @@
       <c r="F14" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="H14" s="40" t="s">
+      <c r="H14" s="2" t="s">
         <v>27</v>
       </c>
     </row>
@@ -4379,7 +4404,47 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>260</v>
+      </c>
+      <c r="B17" t="s">
+        <v>259</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>16</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>262</v>
+      </c>
+      <c r="B18" t="s">
+        <v>264</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18">
+        <v>16</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>164</v>
       </c>
@@ -4430,7 +4495,7 @@
       <c r="D2" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E2" s="45" t="s">
+      <c r="E2" s="48" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4447,7 +4512,7 @@
       <c r="D3" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="45"/>
+      <c r="E3" s="48"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -4462,7 +4527,7 @@
       <c r="D4" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="46" t="s">
+      <c r="E4" s="49" t="s">
         <v>57</v>
       </c>
     </row>
@@ -4479,7 +4544,7 @@
       <c r="D5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="E5" s="46"/>
+      <c r="E5" s="49"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -4494,7 +4559,7 @@
       <c r="D6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="43" t="s">
+      <c r="E6" s="46" t="s">
         <v>58</v>
       </c>
     </row>
@@ -4511,7 +4576,7 @@
       <c r="D7" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E7" s="43"/>
+      <c r="E7" s="46"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -4526,7 +4591,7 @@
       <c r="D8" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="43"/>
+      <c r="E8" s="46"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -4541,7 +4606,7 @@
       <c r="D9" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="44" t="s">
+      <c r="E9" s="47" t="s">
         <v>59</v>
       </c>
     </row>
@@ -4558,7 +4623,7 @@
       <c r="D10" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E10" s="44"/>
+      <c r="E10" s="47"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -4573,7 +4638,7 @@
       <c r="D11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="44"/>
+      <c r="E11" s="47"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="17"/>
@@ -4595,7 +4660,7 @@
       <c r="D13" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="E13" s="45" t="s">
+      <c r="E13" s="48" t="s">
         <v>62</v>
       </c>
     </row>
@@ -4612,7 +4677,7 @@
       <c r="D14" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="E14" s="45"/>
+      <c r="E14" s="48"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -4627,7 +4692,7 @@
       <c r="D15" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="46" t="s">
+      <c r="E15" s="49" t="s">
         <v>71</v>
       </c>
     </row>
@@ -4644,7 +4709,7 @@
       <c r="D16" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="E16" s="46"/>
+      <c r="E16" s="49"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
@@ -4659,7 +4724,7 @@
       <c r="D17" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E17" s="43" t="s">
+      <c r="E17" s="46" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4676,7 +4741,7 @@
       <c r="D18" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E18" s="43"/>
+      <c r="E18" s="46"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
@@ -4691,7 +4756,7 @@
       <c r="D19" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E19" s="43"/>
+      <c r="E19" s="46"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
@@ -4706,7 +4771,7 @@
       <c r="D20" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="44" t="s">
+      <c r="E20" s="47" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4723,7 +4788,7 @@
       <c r="D21" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E21" s="44"/>
+      <c r="E21" s="47"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
@@ -4738,7 +4803,7 @@
       <c r="D22" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="E22" s="44"/>
+      <c r="E22" s="47"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="17"/>
@@ -4760,7 +4825,7 @@
       <c r="D24" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E24" s="45" t="s">
+      <c r="E24" s="48" t="s">
         <v>57</v>
       </c>
     </row>
@@ -4777,7 +4842,7 @@
       <c r="D25" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="E25" s="45"/>
+      <c r="E25" s="48"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
@@ -4792,7 +4857,7 @@
       <c r="D26" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E26" s="46" t="s">
+      <c r="E26" s="49" t="s">
         <v>71</v>
       </c>
     </row>
@@ -4809,7 +4874,7 @@
       <c r="D27" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="E27" s="46"/>
+      <c r="E27" s="49"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
@@ -4824,7 +4889,7 @@
       <c r="D28" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="E28" s="43" t="s">
+      <c r="E28" s="46" t="s">
         <v>59</v>
       </c>
     </row>
@@ -4841,7 +4906,7 @@
       <c r="D29" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E29" s="43"/>
+      <c r="E29" s="46"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
@@ -4856,7 +4921,7 @@
       <c r="D30" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E30" s="43"/>
+      <c r="E30" s="46"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
@@ -4871,7 +4936,7 @@
       <c r="D31" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="E31" s="44" t="s">
+      <c r="E31" s="47" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4888,7 +4953,7 @@
       <c r="D32" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E32" s="44"/>
+      <c r="E32" s="47"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
@@ -4903,7 +4968,7 @@
       <c r="D33" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="E33" s="44"/>
+      <c r="E33" s="47"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="17"/>
@@ -4925,7 +4990,7 @@
       <c r="D35" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E35" s="45" t="s">
+      <c r="E35" s="48" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4942,7 +5007,7 @@
       <c r="D36" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="45"/>
+      <c r="E36" s="48"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
@@ -4957,7 +5022,7 @@
       <c r="D37" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="E37" s="46" t="s">
+      <c r="E37" s="49" t="s">
         <v>62</v>
       </c>
     </row>
@@ -4974,7 +5039,7 @@
       <c r="D38" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E38" s="46"/>
+      <c r="E38" s="49"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
@@ -4989,7 +5054,7 @@
       <c r="D39" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E39" s="43" t="s">
+      <c r="E39" s="46" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5006,7 +5071,7 @@
       <c r="D40" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E40" s="43"/>
+      <c r="E40" s="46"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
@@ -5021,7 +5086,7 @@
       <c r="D41" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E41" s="43"/>
+      <c r="E41" s="46"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
@@ -5036,7 +5101,7 @@
       <c r="D42" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E42" s="44" t="s">
+      <c r="E42" s="47" t="s">
         <v>72</v>
       </c>
     </row>
@@ -5053,7 +5118,7 @@
       <c r="D43" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E43" s="44"/>
+      <c r="E43" s="47"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
@@ -5068,26 +5133,26 @@
       <c r="D44" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E44" s="44"/>
+      <c r="E44" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E17:E19"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="E26:E27"/>
     <mergeCell ref="E28:E30"/>
     <mergeCell ref="E31:E33"/>
     <mergeCell ref="E39:E41"/>
     <mergeCell ref="E42:E44"/>
     <mergeCell ref="E35:E36"/>
     <mergeCell ref="E37:E38"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E17:E19"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="E9:E11"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="E13:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5095,10 +5160,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{992A3727-2875-0A4F-9138-C75C5524DA50}">
-  <dimension ref="A1:I187"/>
+  <dimension ref="A1:I204"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="48.6640625" customWidth="1"/>
+    <col min="1" max="1" width="57.5" customWidth="1"/>
     <col min="3" max="3" width="16.33203125" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
     <col min="5" max="5" width="21.83203125" customWidth="1"/>
@@ -5134,7 +5199,7 @@
       <c r="D2" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="45" t="s">
+      <c r="E2" s="48" t="s">
         <v>93</v>
       </c>
     </row>
@@ -5151,7 +5216,7 @@
       <c r="D3" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E3" s="45"/>
+      <c r="E3" s="48"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -5166,7 +5231,7 @@
       <c r="D4" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="E4" s="45"/>
+      <c r="E4" s="48"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -5181,7 +5246,7 @@
       <c r="D5" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="E5" s="49" t="s">
+      <c r="E5" s="56" t="s">
         <v>78</v>
       </c>
     </row>
@@ -5198,7 +5263,7 @@
       <c r="D6" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="49"/>
+      <c r="E6" s="56"/>
       <c r="H6" s="10"/>
       <c r="I6" s="11"/>
     </row>
@@ -5215,7 +5280,7 @@
       <c r="D7" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="E7" s="49"/>
+      <c r="E7" s="56"/>
       <c r="H7" s="10"/>
       <c r="I7" s="11"/>
     </row>
@@ -5232,7 +5297,7 @@
       <c r="D8" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E8" s="44" t="s">
+      <c r="E8" s="47" t="s">
         <v>94</v>
       </c>
       <c r="H8" s="10"/>
@@ -5251,7 +5316,7 @@
       <c r="D9" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E9" s="44"/>
+      <c r="E9" s="47"/>
       <c r="H9" s="10"/>
       <c r="I9" s="11"/>
     </row>
@@ -5268,7 +5333,7 @@
       <c r="D10" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E10" s="44"/>
+      <c r="E10" s="47"/>
       <c r="H10" s="10"/>
       <c r="I10" s="11"/>
     </row>
@@ -5285,7 +5350,7 @@
       <c r="D11" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="E11" s="44"/>
+      <c r="E11" s="47"/>
       <c r="H11" s="10"/>
       <c r="I11" s="11"/>
     </row>
@@ -5302,7 +5367,7 @@
       <c r="D12" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="E12" s="43" t="s">
+      <c r="E12" s="46" t="s">
         <v>91</v>
       </c>
     </row>
@@ -5319,7 +5384,7 @@
       <c r="D13" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="E13" s="43"/>
+      <c r="E13" s="46"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -5334,7 +5399,7 @@
       <c r="D14" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="E14" s="52" t="s">
+      <c r="E14" s="55" t="s">
         <v>79</v>
       </c>
     </row>
@@ -5351,7 +5416,7 @@
       <c r="D15" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="E15" s="52"/>
+      <c r="E15" s="55"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -5366,7 +5431,7 @@
       <c r="D16" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="E16" s="50" t="s">
+      <c r="E16" s="57" t="s">
         <v>92</v>
       </c>
     </row>
@@ -5383,7 +5448,7 @@
       <c r="D17" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="E17" s="50"/>
+      <c r="E17" s="57"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="17"/>
@@ -5405,7 +5470,7 @@
       <c r="D19" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E19" s="45" t="s">
+      <c r="E19" s="48" t="s">
         <v>93</v>
       </c>
     </row>
@@ -5422,7 +5487,7 @@
       <c r="D20" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E20" s="45"/>
+      <c r="E20" s="48"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
@@ -5437,7 +5502,7 @@
       <c r="D21" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="E21" s="45"/>
+      <c r="E21" s="48"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
@@ -5452,7 +5517,7 @@
       <c r="D22" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="E22" s="49" t="s">
+      <c r="E22" s="56" t="s">
         <v>91</v>
       </c>
     </row>
@@ -5469,7 +5534,7 @@
       <c r="D23" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="E23" s="49"/>
+      <c r="E23" s="56"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
@@ -5484,7 +5549,7 @@
       <c r="D24" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E24" s="44" t="s">
+      <c r="E24" s="47" t="s">
         <v>94</v>
       </c>
     </row>
@@ -5501,7 +5566,7 @@
       <c r="D25" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E25" s="44"/>
+      <c r="E25" s="47"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
@@ -5516,7 +5581,7 @@
       <c r="D26" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E26" s="44"/>
+      <c r="E26" s="47"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
@@ -5531,7 +5596,7 @@
       <c r="D27" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="E27" s="44"/>
+      <c r="E27" s="47"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
@@ -5546,7 +5611,7 @@
       <c r="D28" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="E28" s="43" t="s">
+      <c r="E28" s="46" t="s">
         <v>92</v>
       </c>
     </row>
@@ -5563,7 +5628,7 @@
       <c r="D29" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="E29" s="43"/>
+      <c r="E29" s="46"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
@@ -5578,7 +5643,7 @@
       <c r="D30" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="E30" s="52" t="s">
+      <c r="E30" s="55" t="s">
         <v>78</v>
       </c>
     </row>
@@ -5595,7 +5660,7 @@
       <c r="D31" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="E31" s="52"/>
+      <c r="E31" s="55"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
@@ -5610,7 +5675,7 @@
       <c r="D32" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="E32" s="52"/>
+      <c r="E32" s="55"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
@@ -5625,7 +5690,7 @@
       <c r="D33" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="E33" s="50" t="s">
+      <c r="E33" s="57" t="s">
         <v>79</v>
       </c>
     </row>
@@ -5642,7 +5707,7 @@
       <c r="D34" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="E34" s="50"/>
+      <c r="E34" s="57"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="17"/>
@@ -5664,7 +5729,7 @@
       <c r="D36" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="E36" s="45" t="s">
+      <c r="E36" s="48" t="s">
         <v>102</v>
       </c>
     </row>
@@ -5681,7 +5746,7 @@
       <c r="D37" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="E37" s="45"/>
+      <c r="E37" s="48"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
@@ -5696,7 +5761,7 @@
       <c r="D38" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="E38" s="45"/>
+      <c r="E38" s="48"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
@@ -5711,7 +5776,7 @@
       <c r="D39" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="E39" s="49" t="s">
+      <c r="E39" s="56" t="s">
         <v>106</v>
       </c>
     </row>
@@ -5728,7 +5793,7 @@
       <c r="D40" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="E40" s="49"/>
+      <c r="E40" s="56"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
@@ -5743,7 +5808,7 @@
       <c r="D41" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="E41" s="44" t="s">
+      <c r="E41" s="47" t="s">
         <v>109</v>
       </c>
     </row>
@@ -5760,7 +5825,7 @@
       <c r="D42" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E42" s="44"/>
+      <c r="E42" s="47"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
@@ -5775,7 +5840,7 @@
       <c r="D43" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="E43" s="44"/>
+      <c r="E43" s="47"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
@@ -5790,7 +5855,7 @@
       <c r="D44" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="E44" s="43" t="s">
+      <c r="E44" s="46" t="s">
         <v>115</v>
       </c>
     </row>
@@ -5807,7 +5872,7 @@
       <c r="D45" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="E45" s="43"/>
+      <c r="E45" s="46"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
@@ -5822,7 +5887,7 @@
       <c r="D46" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="E46" s="52" t="s">
+      <c r="E46" s="55" t="s">
         <v>119</v>
       </c>
     </row>
@@ -5839,7 +5904,7 @@
       <c r="D47" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="E47" s="52"/>
+      <c r="E47" s="55"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
@@ -5854,7 +5919,7 @@
       <c r="D48" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="E48" s="52"/>
+      <c r="E48" s="55"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
@@ -5869,7 +5934,7 @@
       <c r="D49" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="E49" s="52"/>
+      <c r="E49" s="55"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
@@ -5884,7 +5949,7 @@
       <c r="D50" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="E50" s="50" t="s">
+      <c r="E50" s="57" t="s">
         <v>122</v>
       </c>
     </row>
@@ -5901,7 +5966,7 @@
       <c r="D51" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="E51" s="50"/>
+      <c r="E51" s="57"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" s="17"/>
@@ -5923,7 +5988,7 @@
       <c r="D53" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="E53" s="49" t="s">
+      <c r="E53" s="56" t="s">
         <v>91</v>
       </c>
     </row>
@@ -5940,7 +6005,7 @@
       <c r="D54" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="E54" s="49"/>
+      <c r="E54" s="56"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
@@ -5955,7 +6020,7 @@
       <c r="D55" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E55" s="45" t="s">
+      <c r="E55" s="48" t="s">
         <v>93</v>
       </c>
     </row>
@@ -5972,7 +6037,7 @@
       <c r="D56" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E56" s="45"/>
+      <c r="E56" s="48"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
@@ -5987,7 +6052,7 @@
       <c r="D57" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="E57" s="45"/>
+      <c r="E57" s="48"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
@@ -6002,7 +6067,7 @@
       <c r="D58" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="E58" s="50" t="s">
+      <c r="E58" s="57" t="s">
         <v>79</v>
       </c>
     </row>
@@ -6019,7 +6084,7 @@
       <c r="D59" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="E59" s="50"/>
+      <c r="E59" s="57"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
@@ -6034,7 +6099,7 @@
       <c r="D60" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="E60" s="52" t="s">
+      <c r="E60" s="55" t="s">
         <v>78</v>
       </c>
     </row>
@@ -6051,7 +6116,7 @@
       <c r="D61" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="E61" s="52"/>
+      <c r="E61" s="55"/>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
@@ -6066,7 +6131,7 @@
       <c r="D62" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="E62" s="52"/>
+      <c r="E62" s="55"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
@@ -6081,7 +6146,7 @@
       <c r="D63" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="E63" s="43" t="s">
+      <c r="E63" s="46" t="s">
         <v>92</v>
       </c>
     </row>
@@ -6098,7 +6163,7 @@
       <c r="D64" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="E64" s="43"/>
+      <c r="E64" s="46"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
@@ -6113,7 +6178,7 @@
       <c r="D65" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E65" s="44" t="s">
+      <c r="E65" s="47" t="s">
         <v>94</v>
       </c>
     </row>
@@ -6130,7 +6195,7 @@
       <c r="D66" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E66" s="44"/>
+      <c r="E66" s="47"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
@@ -6145,7 +6210,7 @@
       <c r="D67" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E67" s="44"/>
+      <c r="E67" s="47"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
@@ -6160,7 +6225,7 @@
       <c r="D68" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="E68" s="44"/>
+      <c r="E68" s="47"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" s="17"/>
@@ -6182,7 +6247,7 @@
       <c r="D70" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="E70" s="49" t="s">
+      <c r="E70" s="56" t="s">
         <v>91</v>
       </c>
     </row>
@@ -6199,7 +6264,7 @@
       <c r="D71" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="E71" s="49"/>
+      <c r="E71" s="56"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
@@ -6214,7 +6279,7 @@
       <c r="D72" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E72" s="45" t="s">
+      <c r="E72" s="48" t="s">
         <v>93</v>
       </c>
     </row>
@@ -6231,7 +6296,7 @@
       <c r="D73" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E73" s="45"/>
+      <c r="E73" s="48"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
@@ -6246,7 +6311,7 @@
       <c r="D74" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="E74" s="45"/>
+      <c r="E74" s="48"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
@@ -6261,7 +6326,7 @@
       <c r="D75" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="E75" s="50" t="s">
+      <c r="E75" s="57" t="s">
         <v>79</v>
       </c>
     </row>
@@ -6278,7 +6343,7 @@
       <c r="D76" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="E76" s="50"/>
+      <c r="E76" s="57"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
@@ -6293,7 +6358,7 @@
       <c r="D77" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="E77" s="52" t="s">
+      <c r="E77" s="55" t="s">
         <v>78</v>
       </c>
     </row>
@@ -6310,7 +6375,7 @@
       <c r="D78" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="E78" s="52"/>
+      <c r="E78" s="55"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
@@ -6325,7 +6390,7 @@
       <c r="D79" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="E79" s="52"/>
+      <c r="E79" s="55"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
@@ -6340,7 +6405,7 @@
       <c r="D80" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="E80" s="43" t="s">
+      <c r="E80" s="46" t="s">
         <v>92</v>
       </c>
     </row>
@@ -6357,7 +6422,7 @@
       <c r="D81" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="E81" s="43"/>
+      <c r="E81" s="46"/>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
@@ -6372,7 +6437,7 @@
       <c r="D82" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E82" s="44" t="s">
+      <c r="E82" s="47" t="s">
         <v>94</v>
       </c>
     </row>
@@ -6389,7 +6454,7 @@
       <c r="D83" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E83" s="44"/>
+      <c r="E83" s="47"/>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
@@ -6404,7 +6469,7 @@
       <c r="D84" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E84" s="44"/>
+      <c r="E84" s="47"/>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
@@ -6419,7 +6484,7 @@
       <c r="D85" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="E85" s="44"/>
+      <c r="E85" s="47"/>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86" s="17"/>
@@ -6441,7 +6506,7 @@
       <c r="D87" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E87" s="45" t="s">
+      <c r="E87" s="48" t="s">
         <v>93</v>
       </c>
     </row>
@@ -6458,7 +6523,7 @@
       <c r="D88" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E88" s="45"/>
+      <c r="E88" s="48"/>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
@@ -6473,7 +6538,7 @@
       <c r="D89" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="E89" s="45"/>
+      <c r="E89" s="48"/>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
@@ -6488,7 +6553,7 @@
       <c r="D90" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="E90" s="49" t="s">
+      <c r="E90" s="56" t="s">
         <v>91</v>
       </c>
       <c r="H90" s="10"/>
@@ -6507,7 +6572,7 @@
       <c r="D91" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="E91" s="49"/>
+      <c r="E91" s="56"/>
       <c r="H91" s="10"/>
       <c r="I91" s="11"/>
     </row>
@@ -6524,7 +6589,7 @@
       <c r="D92" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E92" s="44" t="s">
+      <c r="E92" s="47" t="s">
         <v>94</v>
       </c>
       <c r="H92" s="10"/>
@@ -6543,7 +6608,7 @@
       <c r="D93" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E93" s="44"/>
+      <c r="E93" s="47"/>
       <c r="H93" s="10"/>
       <c r="I93" s="11"/>
     </row>
@@ -6560,7 +6625,7 @@
       <c r="D94" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E94" s="44"/>
+      <c r="E94" s="47"/>
       <c r="H94" s="10"/>
       <c r="I94" s="11"/>
     </row>
@@ -6577,7 +6642,7 @@
       <c r="D95" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="E95" s="44"/>
+      <c r="E95" s="47"/>
       <c r="H95" s="10"/>
       <c r="I95" s="11"/>
     </row>
@@ -6594,7 +6659,7 @@
       <c r="D96" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="E96" s="43" t="s">
+      <c r="E96" s="46" t="s">
         <v>92</v>
       </c>
     </row>
@@ -6611,7 +6676,7 @@
       <c r="D97" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="E97" s="43"/>
+      <c r="E97" s="46"/>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
@@ -6626,7 +6691,7 @@
       <c r="D98" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="E98" s="52" t="s">
+      <c r="E98" s="55" t="s">
         <v>78</v>
       </c>
     </row>
@@ -6643,7 +6708,7 @@
       <c r="D99" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="E99" s="52"/>
+      <c r="E99" s="55"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
@@ -6658,7 +6723,7 @@
       <c r="D100" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="E100" s="52"/>
+      <c r="E100" s="55"/>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
@@ -6673,7 +6738,7 @@
       <c r="D101" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="E101" s="50" t="s">
+      <c r="E101" s="57" t="s">
         <v>79</v>
       </c>
     </row>
@@ -6690,7 +6755,7 @@
       <c r="D102" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="E102" s="50"/>
+      <c r="E102" s="57"/>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" s="17"/>
@@ -6712,7 +6777,7 @@
       <c r="D104" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="E104" s="47" t="s">
+      <c r="E104" s="51" t="s">
         <v>157</v>
       </c>
     </row>
@@ -6729,7 +6794,7 @@
       <c r="D105" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="E105" s="47"/>
+      <c r="E105" s="51"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
@@ -6744,7 +6809,7 @@
       <c r="D106" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="E106" s="47"/>
+      <c r="E106" s="51"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
@@ -6759,7 +6824,7 @@
       <c r="D107" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="E107" s="51" t="s">
+      <c r="E107" s="52" t="s">
         <v>158</v>
       </c>
     </row>
@@ -6776,7 +6841,7 @@
       <c r="D108" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="E108" s="51"/>
+      <c r="E108" s="52"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
@@ -6791,7 +6856,7 @@
       <c r="D109" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="E109" s="51"/>
+      <c r="E109" s="52"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
@@ -6806,7 +6871,7 @@
       <c r="D110" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="E110" s="51"/>
+      <c r="E110" s="52"/>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
@@ -6821,7 +6886,7 @@
       <c r="D111" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="E111" s="51"/>
+      <c r="E111" s="52"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
@@ -6967,7 +7032,7 @@
       <c r="D121" s="27" t="s">
         <v>168</v>
       </c>
-      <c r="E121" s="43" t="s">
+      <c r="E121" s="46" t="s">
         <v>180</v>
       </c>
     </row>
@@ -6984,7 +7049,7 @@
       <c r="D122" s="27" t="s">
         <v>169</v>
       </c>
-      <c r="E122" s="43"/>
+      <c r="E122" s="46"/>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
@@ -6999,7 +7064,7 @@
       <c r="D123" s="27" t="s">
         <v>170</v>
       </c>
-      <c r="E123" s="43"/>
+      <c r="E123" s="46"/>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
@@ -7014,7 +7079,7 @@
       <c r="D124" s="27" t="s">
         <v>171</v>
       </c>
-      <c r="E124" s="43"/>
+      <c r="E124" s="46"/>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
@@ -7029,7 +7094,7 @@
       <c r="D125" s="28" t="s">
         <v>172</v>
       </c>
-      <c r="E125" s="49" t="s">
+      <c r="E125" s="56" t="s">
         <v>181</v>
       </c>
     </row>
@@ -7046,7 +7111,7 @@
       <c r="D126" s="28" t="s">
         <v>173</v>
       </c>
-      <c r="E126" s="49"/>
+      <c r="E126" s="56"/>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
@@ -7061,7 +7126,7 @@
       <c r="D127" s="28" t="s">
         <v>174</v>
       </c>
-      <c r="E127" s="49"/>
+      <c r="E127" s="56"/>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
@@ -7076,7 +7141,7 @@
       <c r="D128" s="28" t="s">
         <v>175</v>
       </c>
-      <c r="E128" s="49"/>
+      <c r="E128" s="56"/>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
@@ -7108,7 +7173,7 @@
       <c r="D130" s="31" t="s">
         <v>176</v>
       </c>
-      <c r="E130" s="47" t="s">
+      <c r="E130" s="51" t="s">
         <v>190</v>
       </c>
     </row>
@@ -7125,7 +7190,7 @@
       <c r="D131" s="31" t="s">
         <v>178</v>
       </c>
-      <c r="E131" s="47"/>
+      <c r="E131" s="51"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
@@ -7140,7 +7205,7 @@
       <c r="D132" s="31" t="s">
         <v>179</v>
       </c>
-      <c r="E132" s="47"/>
+      <c r="E132" s="51"/>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
@@ -7218,7 +7283,7 @@
       <c r="D138" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="E138" s="47" t="s">
+      <c r="E138" s="51" t="s">
         <v>212</v>
       </c>
     </row>
@@ -7235,7 +7300,7 @@
       <c r="D139" s="20" t="s">
         <v>197</v>
       </c>
-      <c r="E139" s="47"/>
+      <c r="E139" s="51"/>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
@@ -7250,7 +7315,7 @@
       <c r="D140" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="E140" s="47"/>
+      <c r="E140" s="51"/>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
@@ -7265,7 +7330,7 @@
       <c r="D141" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="E141" s="47"/>
+      <c r="E141" s="51"/>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
@@ -7280,7 +7345,7 @@
       <c r="D142" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="E142" s="51" t="s">
+      <c r="E142" s="52" t="s">
         <v>213</v>
       </c>
     </row>
@@ -7297,7 +7362,7 @@
       <c r="D143" s="21" t="s">
         <v>201</v>
       </c>
-      <c r="E143" s="51"/>
+      <c r="E143" s="52"/>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
@@ -7312,7 +7377,7 @@
       <c r="D144" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="E144" s="51"/>
+      <c r="E144" s="52"/>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
@@ -7327,7 +7392,7 @@
       <c r="D145" s="21" t="s">
         <v>203</v>
       </c>
-      <c r="E145" s="51"/>
+      <c r="E145" s="52"/>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
@@ -7473,7 +7538,7 @@
       <c r="D155" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="E155" s="43" t="s">
+      <c r="E155" s="46" t="s">
         <v>91</v>
       </c>
     </row>
@@ -7490,7 +7555,7 @@
       <c r="D156" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="E156" s="43"/>
+      <c r="E156" s="46"/>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
@@ -7505,7 +7570,7 @@
       <c r="D157" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="E157" s="46" t="s">
+      <c r="E157" s="49" t="s">
         <v>93</v>
       </c>
     </row>
@@ -7522,7 +7587,7 @@
       <c r="D158" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="E158" s="46"/>
+      <c r="E158" s="49"/>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
@@ -7537,7 +7602,7 @@
       <c r="D159" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="E159" s="46"/>
+      <c r="E159" s="49"/>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
@@ -7552,7 +7617,7 @@
       <c r="D160" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="E160" s="45" t="s">
+      <c r="E160" s="48" t="s">
         <v>79</v>
       </c>
       <c r="G160" s="10"/>
@@ -7571,7 +7636,7 @@
       <c r="D161" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="E161" s="45"/>
+      <c r="E161" s="48"/>
       <c r="G161" s="10"/>
       <c r="H161" s="11"/>
     </row>
@@ -7588,7 +7653,7 @@
       <c r="D162" s="36" t="s">
         <v>88</v>
       </c>
-      <c r="E162" s="47" t="s">
+      <c r="E162" s="51" t="s">
         <v>78</v>
       </c>
       <c r="G162" s="10"/>
@@ -7607,7 +7672,7 @@
       <c r="D163" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="E163" s="47"/>
+      <c r="E163" s="51"/>
       <c r="G163" s="10"/>
       <c r="H163" s="11"/>
     </row>
@@ -7624,7 +7689,7 @@
       <c r="D164" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="E164" s="47"/>
+      <c r="E164" s="51"/>
       <c r="G164" s="10"/>
       <c r="H164" s="11"/>
     </row>
@@ -7641,7 +7706,7 @@
       <c r="D165" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="E165" s="44" t="s">
+      <c r="E165" s="47" t="s">
         <v>92</v>
       </c>
       <c r="G165" s="10"/>
@@ -7660,7 +7725,7 @@
       <c r="D166" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="E166" s="44"/>
+      <c r="E166" s="47"/>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
@@ -7675,7 +7740,7 @@
       <c r="D167" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="E167" s="48" t="s">
+      <c r="E167" s="50" t="s">
         <v>94</v>
       </c>
     </row>
@@ -7692,7 +7757,7 @@
       <c r="D168" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E168" s="48"/>
+      <c r="E168" s="50"/>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
@@ -7707,7 +7772,7 @@
       <c r="D169" s="38" t="s">
         <v>87</v>
       </c>
-      <c r="E169" s="48"/>
+      <c r="E169" s="50"/>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
@@ -7722,13 +7787,13 @@
       <c r="D170" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="E170" s="48"/>
+      <c r="E170" s="50"/>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A171" s="17"/>
       <c r="B171" s="17"/>
       <c r="C171" s="17"/>
-      <c r="D171" s="39"/>
+      <c r="D171" s="17"/>
       <c r="E171" s="17"/>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.2">
@@ -7744,7 +7809,7 @@
       <c r="D172" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="E172" s="43" t="s">
+      <c r="E172" s="46" t="s">
         <v>91</v>
       </c>
     </row>
@@ -7761,7 +7826,7 @@
       <c r="D173" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="E173" s="43"/>
+      <c r="E173" s="46"/>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
@@ -7776,7 +7841,7 @@
       <c r="D174" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="E174" s="46" t="s">
+      <c r="E174" s="49" t="s">
         <v>93</v>
       </c>
     </row>
@@ -7793,7 +7858,7 @@
       <c r="D175" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="E175" s="46"/>
+      <c r="E175" s="49"/>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
@@ -7808,7 +7873,7 @@
       <c r="D176" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="E176" s="46"/>
+      <c r="E176" s="49"/>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
@@ -7823,7 +7888,7 @@
       <c r="D177" s="34" t="s">
         <v>221</v>
       </c>
-      <c r="E177" s="46"/>
+      <c r="E177" s="49"/>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
@@ -7838,7 +7903,7 @@
       <c r="D178" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="E178" s="45" t="s">
+      <c r="E178" s="48" t="s">
         <v>79</v>
       </c>
     </row>
@@ -7855,7 +7920,7 @@
       <c r="D179" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="E179" s="45"/>
+      <c r="E179" s="48"/>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
@@ -7870,7 +7935,7 @@
       <c r="D180" s="36" t="s">
         <v>88</v>
       </c>
-      <c r="E180" s="47" t="s">
+      <c r="E180" s="51" t="s">
         <v>78</v>
       </c>
     </row>
@@ -7887,7 +7952,7 @@
       <c r="D181" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="E181" s="47"/>
+      <c r="E181" s="51"/>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
@@ -7902,7 +7967,7 @@
       <c r="D182" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="E182" s="47"/>
+      <c r="E182" s="51"/>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
@@ -7917,7 +7982,7 @@
       <c r="D183" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="E183" s="44" t="s">
+      <c r="E183" s="47" t="s">
         <v>92</v>
       </c>
     </row>
@@ -7934,7 +7999,7 @@
       <c r="D184" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="E184" s="44"/>
+      <c r="E184" s="47"/>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
@@ -7949,7 +8014,7 @@
       <c r="D185" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="E185" s="48" t="s">
+      <c r="E185" s="50" t="s">
         <v>94</v>
       </c>
     </row>
@@ -7966,7 +8031,7 @@
       <c r="D186" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E186" s="48"/>
+      <c r="E186" s="50"/>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
@@ -7981,47 +8046,277 @@
       <c r="D187" s="38" t="s">
         <v>87</v>
       </c>
-      <c r="E187" s="48"/>
+      <c r="E187" s="50"/>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A188" s="17"/>
+      <c r="B188" s="17"/>
+      <c r="C188" s="17"/>
+      <c r="D188" s="17"/>
+      <c r="E188" s="17"/>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A189" t="s">
+        <v>259</v>
+      </c>
+      <c r="B189" s="2">
+        <v>1</v>
+      </c>
+      <c r="C189" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D189" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="E189" s="49" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A190" t="s">
+        <v>259</v>
+      </c>
+      <c r="B190" s="2">
+        <v>2</v>
+      </c>
+      <c r="C190" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D190" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="E190" s="49"/>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A191" t="s">
+        <v>259</v>
+      </c>
+      <c r="B191" s="2">
+        <v>3</v>
+      </c>
+      <c r="C191" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D191" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="E191" s="49"/>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A192" t="s">
+        <v>259</v>
+      </c>
+      <c r="B192" s="2">
+        <v>4</v>
+      </c>
+      <c r="C192" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D192" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="E192" s="51" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A193" t="s">
+        <v>259</v>
+      </c>
+      <c r="B193" s="2">
+        <v>5</v>
+      </c>
+      <c r="C193" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D193" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="E193" s="51"/>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A194" t="s">
+        <v>259</v>
+      </c>
+      <c r="B194" s="2">
+        <v>6</v>
+      </c>
+      <c r="C194" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D194" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="E194" s="51"/>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A195" t="s">
+        <v>259</v>
+      </c>
+      <c r="B195" s="2">
+        <v>7</v>
+      </c>
+      <c r="C195" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D195" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="E195" s="50" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A196" t="s">
+        <v>259</v>
+      </c>
+      <c r="B196" s="2">
+        <v>8</v>
+      </c>
+      <c r="C196" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D196" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="E196" s="50"/>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A197" t="s">
+        <v>259</v>
+      </c>
+      <c r="B197" s="2">
+        <v>9</v>
+      </c>
+      <c r="C197" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D197" s="38" t="s">
+        <v>87</v>
+      </c>
+      <c r="E197" s="50"/>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A198" t="s">
+        <v>259</v>
+      </c>
+      <c r="B198" s="2">
+        <v>10</v>
+      </c>
+      <c r="C198" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D198" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="E198" s="46" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A199" t="s">
+        <v>259</v>
+      </c>
+      <c r="B199" s="2">
+        <v>11</v>
+      </c>
+      <c r="C199" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D199" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="E199" s="46"/>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A200" t="s">
+        <v>259</v>
+      </c>
+      <c r="B200" s="2">
+        <v>12</v>
+      </c>
+      <c r="C200" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D200" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="E200" s="48" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A201" t="s">
+        <v>259</v>
+      </c>
+      <c r="B201" s="2">
+        <v>13</v>
+      </c>
+      <c r="C201" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D201" s="35" t="s">
+        <v>81</v>
+      </c>
+      <c r="E201" s="48"/>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A202" t="s">
+        <v>259</v>
+      </c>
+      <c r="B202" s="2">
+        <v>14</v>
+      </c>
+      <c r="C202" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D202" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="E202" s="47" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A203" t="s">
+        <v>259</v>
+      </c>
+      <c r="B203" s="2">
+        <v>15</v>
+      </c>
+      <c r="C203" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D203" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="E203" s="47"/>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A204" t="s">
+        <v>259</v>
+      </c>
+      <c r="B204" s="2">
+        <v>16</v>
+      </c>
+      <c r="C204" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D204" s="36" t="s">
+        <v>258</v>
+      </c>
+      <c r="E204" s="45" t="s">
+        <v>78</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="59">
-    <mergeCell ref="E167:E170"/>
-    <mergeCell ref="E155:E156"/>
-    <mergeCell ref="E157:E159"/>
-    <mergeCell ref="E160:E161"/>
-    <mergeCell ref="E162:E164"/>
-    <mergeCell ref="E165:E166"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="E150:E153"/>
-    <mergeCell ref="E130:E132"/>
-    <mergeCell ref="E41:E43"/>
-    <mergeCell ref="E44:E45"/>
-    <mergeCell ref="E46:E49"/>
-    <mergeCell ref="E55:E57"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="E121:E124"/>
-    <mergeCell ref="E125:E128"/>
-    <mergeCell ref="E112:E114"/>
-    <mergeCell ref="E115:E119"/>
-    <mergeCell ref="E65:E68"/>
-    <mergeCell ref="E82:E85"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="E77:E79"/>
-    <mergeCell ref="E80:E81"/>
-    <mergeCell ref="E101:E102"/>
-    <mergeCell ref="E87:E89"/>
-    <mergeCell ref="E90:E91"/>
-    <mergeCell ref="E92:E95"/>
-    <mergeCell ref="E96:E97"/>
-    <mergeCell ref="E98:E100"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E14:E15"/>
+  <mergeCells count="65">
+    <mergeCell ref="E180:E182"/>
+    <mergeCell ref="E183:E184"/>
+    <mergeCell ref="E185:E187"/>
+    <mergeCell ref="E172:E173"/>
+    <mergeCell ref="E174:E177"/>
+    <mergeCell ref="E178:E179"/>
     <mergeCell ref="E22:E23"/>
     <mergeCell ref="E19:E21"/>
     <mergeCell ref="E33:E34"/>
@@ -8038,12 +8333,49 @@
     <mergeCell ref="E50:E51"/>
     <mergeCell ref="E63:E64"/>
     <mergeCell ref="E60:E62"/>
-    <mergeCell ref="E180:E182"/>
-    <mergeCell ref="E183:E184"/>
-    <mergeCell ref="E185:E187"/>
-    <mergeCell ref="E172:E173"/>
-    <mergeCell ref="E174:E177"/>
-    <mergeCell ref="E178:E179"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="E121:E124"/>
+    <mergeCell ref="E125:E128"/>
+    <mergeCell ref="E112:E114"/>
+    <mergeCell ref="E115:E119"/>
+    <mergeCell ref="E65:E68"/>
+    <mergeCell ref="E82:E85"/>
+    <mergeCell ref="E75:E76"/>
+    <mergeCell ref="E77:E79"/>
+    <mergeCell ref="E80:E81"/>
+    <mergeCell ref="E101:E102"/>
+    <mergeCell ref="E87:E89"/>
+    <mergeCell ref="E90:E91"/>
+    <mergeCell ref="E92:E95"/>
+    <mergeCell ref="E96:E97"/>
+    <mergeCell ref="E98:E100"/>
+    <mergeCell ref="E41:E43"/>
+    <mergeCell ref="E44:E45"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="E55:E57"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="E150:E153"/>
+    <mergeCell ref="E130:E132"/>
+    <mergeCell ref="E167:E170"/>
+    <mergeCell ref="E155:E156"/>
+    <mergeCell ref="E157:E159"/>
+    <mergeCell ref="E160:E161"/>
+    <mergeCell ref="E162:E164"/>
+    <mergeCell ref="E165:E166"/>
+    <mergeCell ref="E202:E203"/>
+    <mergeCell ref="E195:E197"/>
+    <mergeCell ref="E198:E199"/>
+    <mergeCell ref="E189:E191"/>
+    <mergeCell ref="E192:E194"/>
+    <mergeCell ref="E200:E201"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8066,60 +8398,60 @@
   <sheetData>
     <row r="1" spans="2:4" ht="24" x14ac:dyDescent="0.3">
       <c r="B1" s="63" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C1" s="63"/>
       <c r="D1" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="2:4" ht="24" x14ac:dyDescent="0.3">
-      <c r="B2" s="66" t="s">
-        <v>250</v>
-      </c>
-      <c r="C2" s="67"/>
+      <c r="B2" s="58" t="s">
+        <v>247</v>
+      </c>
+      <c r="C2" s="59"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="61" t="s">
         <v>233</v>
       </c>
-      <c r="C3" s="57"/>
+      <c r="C3" s="61"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B4" s="57" t="s">
+      <c r="B4" s="61" t="s">
         <v>234</v>
       </c>
-      <c r="C4" s="57"/>
+      <c r="C4" s="61"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B5" s="57" t="s">
+      <c r="B5" s="61" t="s">
         <v>235</v>
       </c>
-      <c r="C5" s="57"/>
+      <c r="C5" s="61"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B6" s="57" t="s">
+      <c r="B6" s="61" t="s">
         <v>236</v>
       </c>
-      <c r="C6" s="57"/>
+      <c r="C6" s="61"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B7" s="57" t="s">
+      <c r="B7" s="61" t="s">
         <v>237</v>
       </c>
-      <c r="C7" s="57"/>
+      <c r="C7" s="61"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B8" s="57" t="s">
-        <v>238</v>
-      </c>
-      <c r="C8" s="57"/>
+      <c r="B8" s="61" t="s">
+        <v>265</v>
+      </c>
+      <c r="C8" s="61"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B9" s="57" t="s">
-        <v>243</v>
-      </c>
-      <c r="C9" s="57"/>
+      <c r="B9" s="61" t="s">
+        <v>242</v>
+      </c>
+      <c r="C9" s="61"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B10" s="4" t="s">
@@ -8130,7 +8462,7 @@
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B11" s="58" t="s">
+      <c r="B11" s="41" t="s">
         <v>28</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -8138,7 +8470,7 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B12" s="58" t="s">
+      <c r="B12" s="41" t="s">
         <v>224</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -8146,7 +8478,7 @@
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B13" s="58" t="s">
+      <c r="B13" s="41" t="s">
         <v>182</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -8154,15 +8486,15 @@
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B14" s="58" t="s">
+      <c r="B14" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="41" t="s">
+      <c r="C14" s="2" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B15" s="58" t="s">
+      <c r="B15" s="41" t="s">
         <v>26</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -8170,7 +8502,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B16" s="58" t="s">
+      <c r="B16" s="41" t="s">
         <v>29</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -8178,7 +8510,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" s="58" t="s">
+      <c r="B17" s="41" t="s">
         <v>33</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -8186,18 +8518,18 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>248</v>
+      <c r="C18" s="2">
+        <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>249</v>
+        <v>266</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B19" s="58" t="s">
+      <c r="B19" s="41" t="s">
         <v>185</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -8205,7 +8537,7 @@
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B20" s="58" t="s">
+      <c r="B20" s="41" t="s">
         <v>31</v>
       </c>
       <c r="C20" s="2">
@@ -8213,7 +8545,7 @@
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B21" s="58" t="s">
+      <c r="B21" s="41" t="s">
         <v>183</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -8221,7 +8553,7 @@
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B22" s="58" t="s">
+      <c r="B22" s="41" t="s">
         <v>188</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -8229,7 +8561,7 @@
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B23" s="59" t="s">
+      <c r="B23" s="42" t="s">
         <v>186</v>
       </c>
       <c r="C23" s="26" t="s">
@@ -8237,7 +8569,7 @@
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B24" s="59" t="s">
+      <c r="B24" s="42" t="s">
         <v>187</v>
       </c>
       <c r="C24" s="26" t="s">
@@ -8245,7 +8577,7 @@
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B25" s="58" t="s">
+      <c r="B25" s="41" t="s">
         <v>228</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -8253,66 +8585,66 @@
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B26" s="55"/>
-      <c r="C26" s="56"/>
+      <c r="B26" s="39"/>
+      <c r="C26" s="40"/>
     </row>
     <row r="27" spans="2:4" ht="24" x14ac:dyDescent="0.3">
-      <c r="B27" s="66" t="s">
-        <v>251</v>
-      </c>
-      <c r="C27" s="67"/>
+      <c r="B27" s="58" t="s">
+        <v>248</v>
+      </c>
+      <c r="C27" s="59"/>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B28" s="64" t="s">
+      <c r="B28" s="60" t="s">
+        <v>238</v>
+      </c>
+      <c r="C28" s="60"/>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B29" s="44" t="s">
         <v>239</v>
       </c>
-      <c r="C28" s="64"/>
-    </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B29" s="65" t="s">
-        <v>240</v>
-      </c>
-      <c r="C29" s="65"/>
+      <c r="C29" s="44"/>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B30" s="60" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C30" s="60"/>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B31" s="60" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C31" s="60"/>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B32" s="57" t="s">
-        <v>242</v>
-      </c>
-      <c r="C32" s="57"/>
+      <c r="B32" s="61" t="s">
+        <v>241</v>
+      </c>
+      <c r="C32" s="61"/>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B33" s="61" t="s">
-        <v>256</v>
-      </c>
-      <c r="C33" s="61"/>
+      <c r="B33" s="43" t="s">
+        <v>253</v>
+      </c>
+      <c r="C33" s="43"/>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B34" s="57" t="s">
+      <c r="B34" s="61" t="s">
+        <v>243</v>
+      </c>
+      <c r="C34" s="61"/>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B35" s="61" t="s">
         <v>244</v>
       </c>
-      <c r="C34" s="57"/>
-    </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B35" s="57" t="s">
-        <v>245</v>
-      </c>
-      <c r="C35" s="57"/>
+      <c r="C35" s="61"/>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B36" s="62" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C36" s="62"/>
       <c r="D36" s="9"/>
@@ -8325,60 +8657,47 @@
       <c r="K36" s="9"/>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B37" s="57" t="s">
-        <v>247</v>
-      </c>
-      <c r="C37" s="57"/>
+      <c r="B37" s="61" t="s">
+        <v>246</v>
+      </c>
+      <c r="C37" s="61"/>
     </row>
     <row r="38" spans="2:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="B38" s="66" t="s">
-        <v>252</v>
-      </c>
-      <c r="C38" s="67"/>
+      <c r="B38" s="58" t="s">
+        <v>249</v>
+      </c>
+      <c r="C38" s="59"/>
     </row>
     <row r="39" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B39" s="65" t="s">
-        <v>253</v>
+      <c r="B39" s="44" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B40" s="60" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C40" s="60"/>
     </row>
     <row r="41" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B41" s="57" t="s">
-        <v>255</v>
-      </c>
-      <c r="C41" s="57"/>
+      <c r="B41" s="61" t="s">
+        <v>252</v>
+      </c>
+      <c r="C41" s="61"/>
     </row>
     <row r="42" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B42" s="57" t="s">
-        <v>256</v>
-      </c>
-      <c r="C42" s="57"/>
+      <c r="B42" s="61" t="s">
+        <v>253</v>
+      </c>
+      <c r="C42" s="61"/>
     </row>
     <row r="43" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B32:C32"/>
@@ -8388,6 +8707,19 @@
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>